<commit_message>
Aktueller Stand: UI aktualisiert, Variablenliste robust, Tabellenoptionen stabil
</commit_message>
<xml_diff>
--- a/TEST ORDNER/ExcelTestDatei1.xlsx
+++ b/TEST ORDNER/ExcelTestDatei1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hubenschmid/ExcelWordVariablen/TEST ORDNER/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46EEB49C-2301-7C4E-82E9-E9E0497571DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0724C3E-01EB-284C-B34E-3D73D74DC83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17220" yWindow="3840" windowWidth="72060" windowHeight="33860" xr2:uid="{9C43E8A6-C309-3444-9A58-F7EF65CA1A49}"/>
+    <workbookView xWindow="14680" yWindow="7900" windowWidth="72060" windowHeight="33860" xr2:uid="{9C43E8A6-C309-3444-9A58-F7EF65CA1A49}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -83,10 +83,31 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF00B0F0"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -176,12 +197,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -189,6 +207,10 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -551,19 +573,19 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2">
-        <v>55</v>
-      </c>
-      <c r="C5" s="2">
-        <v>55</v>
+      <c r="B5" s="6">
+        <v>66</v>
+      </c>
+      <c r="C5" s="5">
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="3">
-        <v>11</v>
-      </c>
-      <c r="C6" s="4">
-        <v>11</v>
+      <c r="B6" s="7">
+        <v>22</v>
+      </c>
+      <c r="C6" s="8">
+        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -571,65 +593,65 @@
         <v>3</v>
       </c>
       <c r="B12" s="1">
-        <v>46344</v>
+        <v>25525</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="5">
-        <v>0.12</v>
+      <c r="B14" s="2">
+        <v>0.77</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="4">
         <v>888</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B20" s="6">
-        <v>999</v>
-      </c>
-      <c r="C20" s="6">
-        <v>999</v>
-      </c>
-      <c r="D20" s="7">
-        <v>99</v>
+      <c r="B20" s="3">
+        <v>1</v>
+      </c>
+      <c r="C20" s="3">
+        <v>1</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B21" s="6">
+      <c r="B21" s="3">
         <v>555</v>
       </c>
-      <c r="C21" s="6">
+      <c r="C21" s="3">
         <v>55</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="4">
         <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="B22" s="6">
+      <c r="B22" s="3">
         <f>SUM(B20:B21)</f>
-        <v>1554</v>
-      </c>
-      <c r="C22" s="6">
+        <v>556</v>
+      </c>
+      <c r="C22" s="3">
         <f t="shared" ref="C22:D22" si="0">SUM(C20:C21)</f>
-        <v>1054</v>
-      </c>
-      <c r="D22" s="7">
+        <v>56</v>
+      </c>
+      <c r="D22" s="4">
         <f t="shared" si="0"/>
-        <v>165</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>